<commit_message>
Update rics.xlsx: 112 valid post-fix ratings, 5 anonymized annotators
Pulled fresh from the live human-eval app. Excluded 71 rows from the
old pre-fix annotator ids (1, 2, 12, 239492, 2204, 2001, 2002,
7564995) -- those predate today's prompt/image-mismatch fix and rate
the wrong image for their prompt, so they'd corrupt a "corrected"
export. Real activity is coming in through the public tunnel now
(guest_* ids).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/results/rics.xlsx
+++ b/data/results/rics.xlsx
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>n = 34 ratings, 1 annotator(s), as of 2026-09-21</t>
+          <t>n = 112 ratings, 5 annotator(s), as of 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -484,22 +484,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="C5" t="n">
-        <v>0.495</v>
+        <v>0.63</v>
       </c>
       <c r="D5" t="n">
-        <v>0.49</v>
+        <v>0.637</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5</v>
+        <v>0.624</v>
       </c>
       <c r="F5" t="n">
-        <v>0.465</v>
+        <v>0.616</v>
       </c>
       <c r="G5" t="n">
-        <v>0.526</v>
+        <v>0.645</v>
       </c>
     </row>
     <row r="6">
@@ -509,22 +509,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>0.616</v>
+        <v>0.707</v>
       </c>
       <c r="D6" t="n">
-        <v>0.637</v>
+        <v>0.727</v>
       </c>
       <c r="E6" t="n">
-        <v>0.649</v>
+        <v>0.711</v>
       </c>
       <c r="F6" t="n">
-        <v>0.628</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>0.549</v>
+        <v>0.696</v>
       </c>
     </row>
     <row r="7">
@@ -534,22 +534,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="C7" t="n">
-        <v>0.444</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>0.41</v>
+        <v>0.541</v>
       </c>
       <c r="E7" t="n">
-        <v>0.543</v>
+        <v>0.596</v>
       </c>
       <c r="F7" t="n">
-        <v>0.433</v>
+        <v>0.553</v>
       </c>
       <c r="G7" t="n">
-        <v>0.39</v>
+        <v>0.5570000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -727,7 +727,7 @@
         <v>0.6</v>
       </c>
       <c r="K3" t="n">
-        <v>0.825</v>
+        <v>0.8250000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -774,7 +774,7 @@
         <v>0.3</v>
       </c>
       <c r="K4" t="n">
-        <v>0.5</v>
+        <v>0.4999999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -1573,7 +1573,7 @@
         <v>0.78</v>
       </c>
       <c r="K21" t="n">
-        <v>0.82</v>
+        <v>0.8200000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -2184,7 +2184,7 @@
         <v>0.7</v>
       </c>
       <c r="K34" t="n">
-        <v>0.525</v>
+        <v>0.5249999999999999</v>
       </c>
     </row>
     <row r="35">
@@ -2232,6 +2232,3672 @@
       </c>
       <c r="K35" t="n">
         <v>0.2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:04</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>poem_0019__FLUX</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>poem_0019</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.675</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:05</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>story_0427__FLUX</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>story_0427</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:11</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>story_0221__FLUX</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>story_0221</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:12</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>story_0263__PixArt</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>story_0263</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.7500000000000001</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:12</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>story_0421__FLUX</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>story_0421</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:10</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>story_0431__SD3</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>story_0431</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:10</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>story_0200__SD3</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>story_0200</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:11</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>story_0405__PixArt</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>story_0405</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:11</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>story_0583__FLUX</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>story_0583</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.6124999999999999</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:12</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>story_0434__FLUX</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>story_0434</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.475</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:13</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>story_0541__FLUX</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>story_0541</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.5875</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:13</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>story_0577__FLUX</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>story_0577</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0.2625</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:14</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>story_0269__PixArt</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>story_0269</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.6125</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:15</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>story_0492__PixArt</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>story_0492</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.6249999999999999</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:15</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>story_0237__FLUX</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>story_0237</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.3374999999999999</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:15</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>story_0251__FLUX</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>story_0251</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.525</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:16</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>story_0276__FLUX</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>story_0276</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0.4875</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:20</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>story_0517__FLUX</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>story_0517</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.775</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:21</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>story_0529__SD3</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>story_0529</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.7125</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:22</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>story_0262__SD3</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>story_0262</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.7875</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:43</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>story_0224__FLUX</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>story_0224</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:44</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>poem_0049__PixArt</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>poem_0049</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:44</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>poem_0112__PixArt</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>poem_0112</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:46</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>poem_0064__PixArt</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>poem_0064</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.775</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:47</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>poem_0117__PixArt</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>poem_0117</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.8500000000000001</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:48</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>story_0547__PixArt</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>story_0547</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0.825</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:48</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>story_0285__SD3</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>story_0285</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:49</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>story_0393__PixArt</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>story_0393</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:49</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>story_0225__PixArt</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>story_0225</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:51</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>poem_0037__SD3</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>poem_0037</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:52</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>story_0426__FLUX</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>story_0426</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" t="n">
+        <v>1</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0.9625</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:52</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>story_0371__PixArt</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>story_0371</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:53</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>poem_0045__SD3</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>poem_0045</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0.3625</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:54</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>story_0535__SD3</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>story_0535</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0.6749999999999999</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:54</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>poem_0027__FLUX</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>poem_0027</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0.6749999999999999</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:55</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>story_0418__FLUX</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>story_0418</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:57</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>poem_0148__FLUX</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>poem_0148</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0.5375</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:57</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>poem_0168__FLUX</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>poem_0168</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0.4875</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:58</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>story_0547__SD3</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>story_0547</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0.9125</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:58</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>story_0290__SD3</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>story_0290</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0.7875</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:59</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>story_0562__SD3</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>story_0562</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0.7375</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:00</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>story_0548__PixArt</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>story_0548</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:01</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>poem_0042__PixArt</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>poem_0042</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:02</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>poem_0083__FLUX</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>poem_0083</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:02</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>story_0357__FLUX</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>story_0357</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0.7125</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:02</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>story_0566__FLUX</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>story_0566</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J81" t="n">
+        <v>1</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0.925</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:04</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>poem_0065__SD3</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>poem_0065</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.6875</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:05</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>story_0349__SD3</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>story_0349</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0.6749999999999999</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:05</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>story_0202__FLUX</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>story_0202</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0.8375</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:06</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>story_0481__PixArt</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>story_0481</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:08</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>poem_0066__SD3</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>poem_0066</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:09</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>story_0333__FLUX</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>story_0333</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I87" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0.675</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:10</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>poem_0035__SD3</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>poem_0035</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I88" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0.3125</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:11</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>story_0433__FLUX</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>story_0433</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I89" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0.6875</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:11</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>story_0206__FLUX</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>story_0206</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0.5375000000000001</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:12</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>story_0292__SD3</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>story_0292</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:13</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>story_0493__PixArt</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>story_0493</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0.7875</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:13</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>story_0518__SD3</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>story_0518</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0.7250000000000001</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:14</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>story_0515__FLUX</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>story_0515</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:16</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>story_0209__FLUX</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>story_0209</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:17</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>story_0412__FLUX</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>story_0412</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J96" t="n">
+        <v>1</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0.9125</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:22</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>poem_0119__SD3</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>poem_0119</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0.4624999999999999</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>story_0302__FLUX</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>story_0302</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0.8999999999999999</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>story_0575__PixArt</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>story_0575</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0.8625</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>story_0240__FLUX</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>story_0240</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0.8999999999999999</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:22</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>story_0556__FLUX</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>story_0556</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0.5625</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>story_0270__FLUX</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>story_0270</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0.7875</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>poem_0052__PixArt</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>poem_0052</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>story_0423__PixArt</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>story_0423</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G104" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0.825</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>story_0361__PixArt</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>story_0361</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I105" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>story_0397__FLUX</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>story_0397</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J106" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0.7875</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>poem_0174__FLUX</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>poem_0174</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G107" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I107" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0.725</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>story_0444__FLUX</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>story_0444</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J108" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K108" t="n">
+        <v>0.7625</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>poem_0024__PixArt</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>poem_0024</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G109" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I109" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J109" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K109" t="n">
+        <v>0.7749999999999999</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>story_0219__SD3</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>story_0219</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I110" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J110" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0.7124999999999999</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:23</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>story_0287__FLUX</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>story_0287</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H111" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I111" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J111" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K111" t="n">
+        <v>0.7125</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:24</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>poem_0130__PixArt</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>poem_0130</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I112" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J112" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K112" t="n">
+        <v>0.7625000000000001</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:24</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>story_0246__SD3</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>story_0246</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix bot-flood vulnerability, exclude confirmed spam from ratings data
A session with no minimum time between submissions was able to post
116 ratings in 16.5 minutes (median 5s apart, many back-to-back at
3-4s) -- not enough time to read a prompt, look at the image, and set
4 scores. Once the app went public with no auth, that was the only
thing stopping automated flooding.

- human_eval.py: reject a submission if it comes in less than 5s
  after this session's last one, with a message asking the rater to
  slow down
- Exclude the confirmed bot session (guest_898a8ec3, 116 rows) from
  rics.xlsx and live_status.py's valid-row counts, same treatment as
  the earlier pre-fix wrong-pairing rows -- raw data on the server is
  untouched, this only affects what counts as valid for analysis

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/results/rics.xlsx
+++ b/data/results/rics.xlsx
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>n = 112 ratings, 5 annotator(s), as of 2026-09-21</t>
+          <t>n = 175 ratings, 4 annotator(s), as of 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -484,22 +484,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="C5" t="n">
-        <v>0.63</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.637</v>
+        <v>0.699</v>
       </c>
       <c r="E5" t="n">
-        <v>0.624</v>
+        <v>0.675</v>
       </c>
       <c r="F5" t="n">
-        <v>0.616</v>
+        <v>0.674</v>
       </c>
       <c r="G5" t="n">
-        <v>0.645</v>
+        <v>0.703</v>
       </c>
     </row>
     <row r="6">
@@ -509,22 +509,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="C6" t="n">
-        <v>0.707</v>
+        <v>0.732</v>
       </c>
       <c r="D6" t="n">
-        <v>0.727</v>
+        <v>0.748</v>
       </c>
       <c r="E6" t="n">
-        <v>0.711</v>
+        <v>0.731</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.717</v>
       </c>
       <c r="G6" t="n">
-        <v>0.696</v>
+        <v>0.731</v>
       </c>
     </row>
     <row r="7">
@@ -534,22 +534,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.649</v>
       </c>
       <c r="D7" t="n">
-        <v>0.541</v>
+        <v>0.635</v>
       </c>
       <c r="E7" t="n">
-        <v>0.596</v>
+        <v>0.666</v>
       </c>
       <c r="F7" t="n">
-        <v>0.553</v>
+        <v>0.643</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.652</v>
       </c>
     </row>
   </sheetData>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3036,7 +3036,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3083,7 +3083,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3130,7 +3130,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5292,74 +5292,74 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-09-21 16:22</t>
+          <t>2026-09-21 16:24</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>story_0556__FLUX</t>
+          <t>poem_0189__PixArt</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>story_0556</t>
+          <t>poem_0189</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>poem</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>FLUX</t>
+          <t>PixArt</t>
         </is>
       </c>
       <c r="G101" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="H101" t="n">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="I101" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="J101" t="n">
-        <v>0.5</v>
+        <v>0.85</v>
       </c>
       <c r="K101" t="n">
-        <v>0.5625</v>
+        <v>0.7625000000000001</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:25</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>story_0270__FLUX</t>
+          <t>poem_0098__FLUX</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>story_0270</t>
+          <t>poem_0098</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>poem</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -5368,40 +5368,40 @@
         </is>
       </c>
       <c r="G102" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="H102" t="n">
-        <v>0.75</v>
+        <v>0.9</v>
       </c>
       <c r="I102" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="J102" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="K102" t="n">
-        <v>0.7875</v>
+        <v>0.9375</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:25</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>poem_0052__PixArt</t>
+          <t>poem_0194__PixArt</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>poem_0052</t>
+          <t>poem_0194</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5415,45 +5415,45 @@
         </is>
       </c>
       <c r="G103" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H103" t="n">
         <v>0.8</v>
       </c>
-      <c r="H103" t="n">
-        <v>0.7</v>
-      </c>
       <c r="I103" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="J103" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K103" t="n">
         <v>0.8</v>
-      </c>
-      <c r="K103" t="n">
-        <v>0.75</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:25</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>story_0423__PixArt</t>
+          <t>poem_0030__PixArt</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>story_0423</t>
+          <t>poem_0030</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>poem</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -5462,40 +5462,40 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="H104" t="n">
         <v>0.75</v>
       </c>
       <c r="I104" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J104" t="n">
         <v>0.9</v>
       </c>
-      <c r="J104" t="n">
-        <v>0.8</v>
-      </c>
       <c r="K104" t="n">
-        <v>0.825</v>
+        <v>0.7999999999999999</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:26</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>story_0361__PixArt</t>
+          <t>story_0321__FLUX</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>story_0361</t>
+          <t>story_0321</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5505,138 +5505,138 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>PixArt</t>
+          <t>FLUX</t>
         </is>
       </c>
       <c r="G105" t="n">
         <v>0.8</v>
       </c>
       <c r="H105" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I105" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="J105" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="K105" t="n">
-        <v>0.75</v>
+        <v>0.825</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:27</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>story_0397__FLUX</t>
+          <t>poem_0062__PixArt</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>story_0397</t>
+          <t>poem_0062</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>poem</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>FLUX</t>
+          <t>PixArt</t>
         </is>
       </c>
       <c r="G106" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="H106" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="I106" t="n">
         <v>0.75</v>
       </c>
       <c r="J106" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="K106" t="n">
-        <v>0.7875</v>
+        <v>0.725</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:27</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>poem_0174__FLUX</t>
+          <t>story_0213__SD3</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>poem_0174</t>
+          <t>story_0213</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>poem</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>FLUX</t>
+          <t>SD3</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="H107" t="n">
-        <v>0.75</v>
+        <v>0.95</v>
       </c>
       <c r="I107" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="J107" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="K107" t="n">
-        <v>0.725</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:27</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>story_0444__FLUX</t>
+          <t>story_0324__PixArt</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>story_0444</t>
+          <t>story_0324</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5646,14 +5646,14 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>FLUX</t>
+          <t>PixArt</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="H108" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="I108" t="n">
         <v>0.75</v>
@@ -5662,75 +5662,75 @@
         <v>0.75</v>
       </c>
       <c r="K108" t="n">
-        <v>0.7625</v>
+        <v>0.725</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:28</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>poem_0024__PixArt</t>
+          <t>story_0205__FLUX</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>poem_0024</t>
+          <t>story_0205</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>poem</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>PixArt</t>
+          <t>FLUX</t>
         </is>
       </c>
       <c r="G109" t="n">
         <v>0.75</v>
       </c>
       <c r="H109" t="n">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="I109" t="n">
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="J109" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="K109" t="n">
-        <v>0.7749999999999999</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:28</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>story_0219__SD3</t>
+          <t>story_0582__FLUX</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>story_0219</t>
+          <t>story_0582</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5740,91 +5740,91 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>SD3</t>
+          <t>FLUX</t>
         </is>
       </c>
       <c r="G110" t="n">
-        <v>0.65</v>
+        <v>0.9</v>
       </c>
       <c r="H110" t="n">
-        <v>0.65</v>
+        <v>0.85</v>
       </c>
       <c r="I110" t="n">
         <v>0.85</v>
       </c>
       <c r="J110" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="K110" t="n">
-        <v>0.7124999999999999</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-09-21 16:23</t>
+          <t>2026-09-21 16:28</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>story_0287__FLUX</t>
+          <t>poem_0048__PixArt</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>story_0287</t>
+          <t>poem_0048</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>poem</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>FLUX</t>
+          <t>PixArt</t>
         </is>
       </c>
       <c r="G111" t="n">
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H111" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I111" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="J111" t="n">
         <v>0.85</v>
       </c>
       <c r="K111" t="n">
-        <v>0.7125</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-09-21 16:24</t>
+          <t>2026-09-21 16:29</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>poem_0130__PixArt</t>
+          <t>poem_0031__FLUX</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>poem_0130</t>
+          <t>poem_0031</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5834,44 +5834,44 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>PixArt</t>
+          <t>FLUX</t>
         </is>
       </c>
       <c r="G112" t="n">
         <v>0.75</v>
       </c>
       <c r="H112" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="I112" t="n">
         <v>0.8</v>
       </c>
       <c r="J112" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="K112" t="n">
-        <v>0.7625000000000001</v>
+        <v>0.7749999999999999</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-09-21 16:24</t>
+          <t>2026-09-21 16:29</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>story_0246__SD3</t>
+          <t>story_0577__FLUX</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>story_0246</t>
+          <t>story_0577</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5881,23 +5881,2984 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0.7625</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:29</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>story_0594__FLUX</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>story_0594</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G114" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K114" t="n">
+        <v>0.725</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:30</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>story_0573__SD3</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>story_0573</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
           <t>SD3</t>
         </is>
       </c>
-      <c r="G113" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H113" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="I113" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="J113" t="n">
+      <c r="G115" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I115" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K115" t="n">
+        <v>0.8875000000000001</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:30</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>story_0310__FLUX</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>story_0310</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G116" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H116" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I116" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K116" t="n">
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:30</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>story_0395__FLUX</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>story_0395</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I117" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J117" t="n">
+        <v>1</v>
+      </c>
+      <c r="K117" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:30</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>story_0375__SD3</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>story_0375</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I118" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J118" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K118" t="n">
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:31</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>story_0365__PixArt</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>story_0365</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G119" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I119" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J119" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K119" t="n">
+        <v>0.8374999999999999</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:32</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>story_0513__PixArt</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>story_0513</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I120" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J120" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K120" t="n">
+        <v>0.6375</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:32</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>poem_0126__PixArt</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>poem_0126</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I121" t="n">
         <v>0.75</v>
       </c>
-      <c r="K113" t="n">
+      <c r="J121" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K121" t="n">
+        <v>0.7250000000000001</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:33</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>poem_0109__PixArt</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>poem_0109</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G122" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H122" t="n">
         <v>0.75</v>
+      </c>
+      <c r="I122" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J122" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K122" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:33</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>poem_0161__FLUX</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>poem_0161</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G123" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I123" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J123" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K123" t="n">
+        <v>0.7875000000000001</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:34</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>poem_0034__FLUX</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>poem_0034</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G124" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I124" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J124" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K124" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:35</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>story_0434__SD3</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>story_0434</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G125" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I125" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J125" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K125" t="n">
+        <v>0.8625</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:37</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>poem_0021__PixArt</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>poem_0021</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G126" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I126" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J126" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K126" t="n">
+        <v>0.8500000000000001</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:37</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>story_0511__FLUX</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>story_0511</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G127" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H127" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I127" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J127" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K127" t="n">
+        <v>0.8250000000000001</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:38</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>story_0332__PixArt</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>story_0332</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I128" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J128" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K128" t="n">
+        <v>0.8875000000000001</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:38</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>poem_0045__PixArt</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>poem_0045</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H129" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I129" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J129" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K129" t="n">
+        <v>0.8625</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:38</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>story_0462__SD3</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>story_0462</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G130" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H130" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I130" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J130" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K130" t="n">
+        <v>0.7250000000000001</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:38</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>story_0492__FLUX</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>story_0492</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H131" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I131" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J131" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K131" t="n">
+        <v>0.8999999999999999</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:39</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>story_0485__PixArt</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>story_0485</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G132" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H132" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I132" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J132" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K132" t="n">
+        <v>0.925</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:39</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>story_0539__FLUX</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>story_0539</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G133" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H133" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I133" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J133" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K133" t="n">
+        <v>0.825</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:39</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>story_0297__FLUX</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>story_0297</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G134" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H134" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I134" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J134" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K134" t="n">
+        <v>0.8625</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:39</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>story_0405__SD3</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>story_0405</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G135" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H135" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I135" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J135" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K135" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:40</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>poem_0139__FLUX</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>poem_0139</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G136" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H136" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I136" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J136" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K136" t="n">
+        <v>0.8749999999999999</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:40</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>story_0306__FLUX</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>story_0306</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G137" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H137" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I137" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J137" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K137" t="n">
+        <v>0.5625</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:40</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>story_0204__FLUX</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>story_0204</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G138" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H138" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I138" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J138" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K138" t="n">
+        <v>0.925</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:40</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>poem_0062__SD3</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>poem_0062</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G139" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H139" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I139" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J139" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K139" t="n">
+        <v>0.9125</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:41</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>story_0233__PixArt</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>story_0233</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G140" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H140" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I140" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J140" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K140" t="n">
+        <v>0.9125</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:41</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>poem_0011__SD3</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>poem_0011</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G141" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H141" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I141" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J141" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K141" t="n">
+        <v>0.6125</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:41</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>story_0516__SD3</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>story_0516</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G142" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H142" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I142" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J142" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K142" t="n">
+        <v>0.8374999999999999</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:42</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>story_0529__SD3</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>story_0529</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G143" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H143" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I143" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J143" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K143" t="n">
+        <v>0.8999999999999999</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:42</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>poem_0047__SD3</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>poem_0047</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G144" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H144" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I144" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J144" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K144" t="n">
+        <v>0.575</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:42</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>story_0583__SD3</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>story_0583</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G145" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H145" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I145" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J145" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K145" t="n">
+        <v>0.7500000000000001</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:42</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>story_0554__FLUX</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>story_0554</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G146" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H146" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I146" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J146" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K146" t="n">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:43</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>story_0382__FLUX</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>story_0382</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G147" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H147" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I147" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J147" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K147" t="n">
+        <v>0.8875000000000001</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:43</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>poem_0121__SD3</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>poem_0121</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G148" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H148" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I148" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J148" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K148" t="n">
+        <v>0.6125</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:43</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>story_0453__FLUX</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>story_0453</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G149" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H149" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I149" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J149" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K149" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:43</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>poem_0071__SD3</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>poem_0071</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G150" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H150" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J150" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K150" t="n">
+        <v>0.7625</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:44</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>story_0418__PixArt</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>story_0418</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G151" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H151" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J151" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K151" t="n">
+        <v>0.8375</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:44</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>story_0352__SD3</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>story_0352</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G152" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H152" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J152" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K152" t="n">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:44</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>story_0289__SD3</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>story_0289</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G153" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H153" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I153" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J153" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K153" t="n">
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:45</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>poem_0059__FLUX</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>poem_0059</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G154" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H154" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J154" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K154" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:45</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>story_0464__PixArt</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>story_0464</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G155" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H155" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I155" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K155" t="n">
+        <v>0.5875</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:49</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>poem_0180__PixArt</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>poem_0180</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G156" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H156" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I156" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J156" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0.5875</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:49</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>story_0326__SD3</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>story_0326</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G157" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H157" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I157" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J157" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K157" t="n">
+        <v>0.7875</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:49</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>poem_0178__FLUX</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>poem_0178</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G158" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H158" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I158" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J158" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K158" t="n">
+        <v>0.425</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:51</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>story_0392__PixArt</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>story_0392</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G159" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H159" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I159" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J159" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K159" t="n">
+        <v>0.7375</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:51</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>poem_0124__PixArt</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>poem_0124</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G160" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H160" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I160" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J160" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K160" t="n">
+        <v>0.7375</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:51</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>story_0533__SD3</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>story_0533</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G161" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H161" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I161" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K161" t="n">
+        <v>0.8375</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:51</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>story_0547__FLUX</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>story_0547</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G162" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H162" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I162" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J162" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K162" t="n">
+        <v>0.8625</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:52</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>story_0470__PixArt</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>story_0470</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G163" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H163" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I163" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J163" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K163" t="n">
+        <v>0.675</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:52</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>story_0502__SD3</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>story_0502</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G164" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H164" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I164" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J164" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K164" t="n">
+        <v>0.475</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:52</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>story_0508__FLUX</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>story_0508</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G165" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H165" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I165" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J165" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K165" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:53</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>story_0599__SD3</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>story_0599</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G166" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H166" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I166" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J166" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K166" t="n">
+        <v>0.8375</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:57</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>poem_0099__FLUX</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>poem_0099</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G167" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H167" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I167" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J167" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K167" t="n">
+        <v>0.6875</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:57</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>story_0540__FLUX</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>story_0540</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G168" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H168" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I168" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J168" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K168" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:57</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>story_0451__SD3</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>story_0451</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G169" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H169" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I169" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J169" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K169" t="n">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:57</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>poem_0052__PixArt</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>poem_0052</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G170" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H170" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I170" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J170" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K170" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:58</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>story_0289__PixArt</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>story_0289</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>PixArt</t>
+        </is>
+      </c>
+      <c r="G171" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H171" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I171" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J171" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K171" t="n">
+        <v>0.8625</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:58</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>story_0590__SD3</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>story_0590</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G172" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H172" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I172" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J172" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K172" t="n">
+        <v>0.6875</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:59</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>story_0372__SD3</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>story_0372</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G173" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H173" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I173" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J173" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K173" t="n">
+        <v>0.575</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-09-21 17:00</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>story_0371__SD3</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>story_0371</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G174" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H174" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I174" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J174" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K174" t="n">
+        <v>0.7124999999999999</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026-09-21 17:00</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>story_0257__SD3</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>story_0257</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>SD3</t>
+        </is>
+      </c>
+      <c r="G175" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H175" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I175" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J175" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K175" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-09-21 17:01</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>poem_0193__FLUX</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>poem_0193</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>poem</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="G176" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H176" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I176" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J176" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K176" t="n">
+        <v>0.5375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>